<commit_message>
Actualizacion automatica SIPREM y Casuistica GUAJIRA
</commit_message>
<xml_diff>
--- a/siprem_latest.xlsx
+++ b/siprem_latest.xlsx
@@ -29,7 +29,7 @@
     <t>FECHA</t>
   </si>
   <si>
-    <t>21/10/2026 a las 08:08:07</t>
+    <t>21/10/2026 a las 08:20:54</t>
   </si>
   <si>
     <t>Num_Lote</t>
@@ -59854,7 +59854,7 @@
         <v>1</v>
       </c>
       <c r="X638" s="4" t="s">
-        <v>1847</v>
+        <v>244</v>
       </c>
       <c r="Y638" s="4"/>
       <c r="Z638" s="4" t="s">
@@ -69800,7 +69800,7 @@
         <v>1</v>
       </c>
       <c r="X768" s="4" t="s">
-        <v>1847</v>
+        <v>244</v>
       </c>
       <c r="Y768" s="4"/>
       <c r="Z768" s="4" t="s">
@@ -72890,7 +72890,7 @@
         <v>2</v>
       </c>
       <c r="X808" s="4" t="s">
-        <v>1847</v>
+        <v>244</v>
       </c>
       <c r="Y808" s="4"/>
       <c r="Z808" s="4" t="s">

</xml_diff>